<commit_message>
chore: publish latest QA report to GitHub Pages
</commit_message>
<xml_diff>
--- a/test_data/Treaties FullDta/Treaties FullDta_Test_Cases.xlsx
+++ b/test_data/Treaties FullDta/Treaties FullDta_Test_Cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -862,6 +862,126 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>FullDta_07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Treaties FullDta</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>A row's 'View' link opens the full treaty document viewer</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>With Australia selected, clicking the Austria row's 'View' link (previously defined in the page object but never clicked by any test) must replace the table with the full document viewer - a 'Contents' sidebar and the treaty pair's title.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in, Australia selected on Full DTA.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Country: Australia, partner: Austria</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Full DTA
+2. Select Australia
+3. Click the Austria row's 'View' link
+4. Verify the document viewer's 'Contents' sidebar and treaty title are shown</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>With Australia selected, clicking the Austria row's 'View' link (previously defined in the page object but never clicked by any test) must replace the table with the full document viewer - a 'Contents' sidebar and the treaty pair's title.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>The Austria row's 'View' link correctly opened the full document viewer.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The 'View' link opens the full document viewer with the correct title and Contents sidebar</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>FullDta_08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Treaties FullDta</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>The document viewer's Export button downloads a real, non-empty PDF</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>With the Austria document viewer open (Australia selected), clicking 'Export as PDF' must trigger a real download with no failure and a non-zero size.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in, Australia selected, Austria's document viewer open.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Country: Australia, partner: Austria</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in, open Full DTA, select Australia
+2. Open the Austria document viewer
+3. Click the 'Export as PDF' button
+4. Verify a real, non-empty PDF download completed</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>With the Austria document viewer open (Australia selected), clicking 'Export as PDF' must trigger a real download with no failure and a non-zero size.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>The Export button downloaded 'Treaty_Australia - Austria.pdf' (92230 bytes) successfully.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The document viewer's Export button downloads a real, non-empty .pdf file with no failure</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>